<commit_message>
new images and renaming some images
</commit_message>
<xml_diff>
--- a/MasterRekaDishData.xlsx
+++ b/MasterRekaDishData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shady\Desktop\repos\value-recipe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6459B8DE-EB8F-4776-BED7-BA5700D2C1B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0B21D23-984C-4412-8642-DA9C3E869D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{E7948A1B-65AD-4BB0-8EC6-16EC14678B9F}"/>
+    <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{E7948A1B-65AD-4BB0-8EC6-16EC14678B9F}"/>
   </bookViews>
   <sheets>
     <sheet name="Ingredients Master List" sheetId="1" r:id="rId1"/>
@@ -495,10 +495,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CD243A6-3128-45AE-AB78-995ED60CA29C}" name="Table1" displayName="Table1" ref="A1:A147" totalsRowShown="0" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CD243A6-3128-45AE-AB78-995ED60CA29C}" name="Table1" displayName="Table1" ref="A1:A147" totalsRowShown="0" dataDxfId="1">
   <autoFilter ref="A1:A147" xr:uid="{6CD243A6-3128-45AE-AB78-995ED60CA29C}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{96714597-BB3B-4C97-ACBE-6770A363FEDB}" name="Ingredient" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{96714597-BB3B-4C97-ACBE-6770A363FEDB}" name="Ingredient" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
new recipes added fixed some minor issues
</commit_message>
<xml_diff>
--- a/MasterRekaDishData.xlsx
+++ b/MasterRekaDishData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shady\Desktop\repos\value-recipe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0B21D23-984C-4412-8642-DA9C3E869D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9006E18A-9719-48FE-B910-A0C0C950AF84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{E7948A1B-65AD-4BB0-8EC6-16EC14678B9F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
   <si>
     <t>Ingredient</t>
   </si>
@@ -50,30 +50,15 @@
     <t>bacon</t>
   </si>
   <si>
-    <t>baking-powder</t>
-  </si>
-  <si>
     <t>bananas</t>
   </si>
   <si>
     <t>basil</t>
   </si>
   <si>
-    <t>bbq-sauce</t>
-  </si>
-  <si>
     <t>beef</t>
   </si>
   <si>
-    <t>bell-pepper</t>
-  </si>
-  <si>
-    <t>black-beans</t>
-  </si>
-  <si>
-    <t>black-pepper</t>
-  </si>
-  <si>
     <t>bread</t>
   </si>
   <si>
@@ -92,24 +77,15 @@
     <t>cabbage</t>
   </si>
   <si>
-    <t>cake-mix</t>
-  </si>
-  <si>
     <t>capers</t>
   </si>
   <si>
     <t>carrot</t>
   </si>
   <si>
-    <t>cayenne-pepper</t>
-  </si>
-  <si>
     <t>celery</t>
   </si>
   <si>
-    <t>cheddar-cheese</t>
-  </si>
-  <si>
     <t>chickpeas</t>
   </si>
   <si>
@@ -122,15 +98,9 @@
     <t>chocolate</t>
   </si>
   <si>
-    <t>chocolate-chips</t>
-  </si>
-  <si>
     <t>cinnamon</t>
   </si>
   <si>
-    <t>cocoa-powder</t>
-  </si>
-  <si>
     <t>coffee</t>
   </si>
   <si>
@@ -140,90 +110,39 @@
     <t>cornstarch</t>
   </si>
   <si>
-    <t>cottage-cheese</t>
-  </si>
-  <si>
     <t>couscous</t>
   </si>
   <si>
-    <t>cracker</t>
-  </si>
-  <si>
-    <t>cream-cheese</t>
-  </si>
-  <si>
     <t>cumin</t>
   </si>
   <si>
     <t>curry</t>
   </si>
   <si>
-    <t>curry-roux</t>
-  </si>
-  <si>
-    <t>dijon-mustard</t>
-  </si>
-  <si>
     <t>eggs</t>
   </si>
   <si>
-    <t>enchilada-sauce</t>
-  </si>
-  <si>
-    <t>feta-cheese</t>
-  </si>
-  <si>
     <t>fish</t>
   </si>
   <si>
     <t>flour</t>
   </si>
   <si>
-    <t>fudge-sauce</t>
-  </si>
-  <si>
-    <t>garam-masala</t>
-  </si>
-  <si>
     <t>garlic</t>
   </si>
   <si>
-    <t>garlic-powder</t>
-  </si>
-  <si>
     <t>ginger</t>
   </si>
   <si>
-    <t>green-onion</t>
-  </si>
-  <si>
     <t>gruyere</t>
   </si>
   <si>
-    <t>ground-beef</t>
-  </si>
-  <si>
     <t>honey</t>
   </si>
   <si>
     <t>horseradish</t>
   </si>
   <si>
-    <t>hot-sauce</t>
-  </si>
-  <si>
-    <t>ice-cream</t>
-  </si>
-  <si>
-    <t>italian-seasoning</t>
-  </si>
-  <si>
-    <t>italian-sausage</t>
-  </si>
-  <si>
-    <t>lasagna-sheets</t>
-  </si>
-  <si>
     <t>lemon</t>
   </si>
   <si>
@@ -233,33 +152,18 @@
     <t>lettuce</t>
   </si>
   <si>
-    <t>liquid-smoke</t>
-  </si>
-  <si>
     <t>lime</t>
   </si>
   <si>
-    <t>maple-syrup</t>
-  </si>
-  <si>
     <t>mascarpone</t>
   </si>
   <si>
     <t>mayonnaise</t>
   </si>
   <si>
-    <t>mixed-veggies</t>
-  </si>
-  <si>
-    <t>mozzarella-cheese</t>
-  </si>
-  <si>
     <t>mushrooms</t>
   </si>
   <si>
-    <t>nacho-cheese</t>
-  </si>
-  <si>
     <t>nutmeg</t>
   </si>
   <si>
@@ -269,9 +173,6 @@
     <t>onion</t>
   </si>
   <si>
-    <t>orange-juice</t>
-  </si>
-  <si>
     <t>oregano</t>
   </si>
   <si>
@@ -284,9 +185,6 @@
     <t>paprika</t>
   </si>
   <si>
-    <t>parmesan-cheese</t>
-  </si>
-  <si>
     <t>parsley</t>
   </si>
   <si>
@@ -299,24 +197,9 @@
     <t>pickles</t>
   </si>
   <si>
-    <t>pizza-dough</t>
-  </si>
-  <si>
-    <t>pinto-beans</t>
-  </si>
-  <si>
     <t>potatoes</t>
   </si>
   <si>
-    <t>powdered-sugar</t>
-  </si>
-  <si>
-    <t>pumpkin-pie-spice</t>
-  </si>
-  <si>
-    <t>pumpkin-puree</t>
-  </si>
-  <si>
     <t>relish</t>
   </si>
   <si>
@@ -338,21 +221,9 @@
     <t>seaweed</t>
   </si>
   <si>
-    <t>sesame-seeds</t>
-  </si>
-  <si>
     <t>shrimp</t>
   </si>
   <si>
-    <t>snow-peas</t>
-  </si>
-  <si>
-    <t>sour-cream</t>
-  </si>
-  <si>
-    <t>soy-sauce</t>
-  </si>
-  <si>
     <t>spinach</t>
   </si>
   <si>
@@ -362,21 +233,9 @@
     <t>sugar</t>
   </si>
   <si>
-    <t>sun-dried-tomatoes</t>
-  </si>
-  <si>
-    <t>taco-seasoning</t>
-  </si>
-  <si>
-    <t>taco-shells</t>
-  </si>
-  <si>
     <t>tarragon</t>
   </si>
   <si>
-    <t>teriyaki-sauce</t>
-  </si>
-  <si>
     <t>thyme</t>
   </si>
   <si>
@@ -386,9 +245,6 @@
     <t>tortilla</t>
   </si>
   <si>
-    <t>tostada-shells</t>
-  </si>
-  <si>
     <t>vanilla</t>
   </si>
   <si>
@@ -404,22 +260,226 @@
     <t>zucchini</t>
   </si>
   <si>
-    <t>peanuts</t>
-  </si>
-  <si>
-    <t>pastry</t>
-  </si>
-  <si>
     <t>wine</t>
   </si>
   <si>
-    <t>yellow-mustard</t>
-  </si>
-  <si>
     <t>milk</t>
   </si>
   <si>
-    <t>whipped-cream</t>
+    <t>apples</t>
+  </si>
+  <si>
+    <t>baking powder</t>
+  </si>
+  <si>
+    <t>baking soda</t>
+  </si>
+  <si>
+    <t>bbq sauce</t>
+  </si>
+  <si>
+    <t>bell pepper</t>
+  </si>
+  <si>
+    <t>black beans</t>
+  </si>
+  <si>
+    <t>black pepper</t>
+  </si>
+  <si>
+    <t>cake mix</t>
+  </si>
+  <si>
+    <t>cayenne pepper</t>
+  </si>
+  <si>
+    <t>cheddar cheese</t>
+  </si>
+  <si>
+    <t>chocolate chips</t>
+  </si>
+  <si>
+    <t>cilantro</t>
+  </si>
+  <si>
+    <t>cocoa powder</t>
+  </si>
+  <si>
+    <t>cottage cheese</t>
+  </si>
+  <si>
+    <t>crackers</t>
+  </si>
+  <si>
+    <t>cream cheese</t>
+  </si>
+  <si>
+    <t>cucumber</t>
+  </si>
+  <si>
+    <t>curry roux</t>
+  </si>
+  <si>
+    <t>daikon</t>
+  </si>
+  <si>
+    <t>dijon mustard</t>
+  </si>
+  <si>
+    <t>eggplant</t>
+  </si>
+  <si>
+    <t>enchilada sauce</t>
+  </si>
+  <si>
+    <t>feta cheese</t>
+  </si>
+  <si>
+    <t>fudge sauce</t>
+  </si>
+  <si>
+    <t>garam masala</t>
+  </si>
+  <si>
+    <t>garlic powder</t>
+  </si>
+  <si>
+    <t>grapes</t>
+  </si>
+  <si>
+    <t>green onion</t>
+  </si>
+  <si>
+    <t>heavy cream</t>
+  </si>
+  <si>
+    <t>hot sauce</t>
+  </si>
+  <si>
+    <t>ice cream</t>
+  </si>
+  <si>
+    <t>italian seasoning</t>
+  </si>
+  <si>
+    <t>ketchup</t>
+  </si>
+  <si>
+    <t>ladyfingers</t>
+  </si>
+  <si>
+    <t>lasagna sheets</t>
+  </si>
+  <si>
+    <t>liquid smoke</t>
+  </si>
+  <si>
+    <t>mango</t>
+  </si>
+  <si>
+    <t>maple syrup</t>
+  </si>
+  <si>
+    <t>marinara sauce</t>
+  </si>
+  <si>
+    <t>mayo</t>
+  </si>
+  <si>
+    <t>mint</t>
+  </si>
+  <si>
+    <t>mixed veggies</t>
+  </si>
+  <si>
+    <t>mozzarella cheese</t>
+  </si>
+  <si>
+    <t>nacho cheese</t>
+  </si>
+  <si>
+    <t>oats</t>
+  </si>
+  <si>
+    <t>olives</t>
+  </si>
+  <si>
+    <t>orange juice</t>
+  </si>
+  <si>
+    <t>parmesan cheese</t>
+  </si>
+  <si>
+    <t>pear</t>
+  </si>
+  <si>
+    <t>pie crust</t>
+  </si>
+  <si>
+    <t>pinto beans</t>
+  </si>
+  <si>
+    <t>pizza dough</t>
+  </si>
+  <si>
+    <t>pork</t>
+  </si>
+  <si>
+    <t>powdered sugar</t>
+  </si>
+  <si>
+    <t>pumpkin pie spice</t>
+  </si>
+  <si>
+    <t>pumpkin puree</t>
+  </si>
+  <si>
+    <t>red pepper flakes</t>
+  </si>
+  <si>
+    <t>sesame seeds</t>
+  </si>
+  <si>
+    <t>snow peas</t>
+  </si>
+  <si>
+    <t>sour cream</t>
+  </si>
+  <si>
+    <t>soy sauce</t>
+  </si>
+  <si>
+    <t>sun dried tomatoes</t>
+  </si>
+  <si>
+    <t>taco seasoning</t>
+  </si>
+  <si>
+    <t>taco shells</t>
+  </si>
+  <si>
+    <t>tapioca pearls</t>
+  </si>
+  <si>
+    <t>teriyaki sauce</t>
+  </si>
+  <si>
+    <t>tomato sauce</t>
+  </si>
+  <si>
+    <t>tostada shells</t>
+  </si>
+  <si>
+    <t>turmeric</t>
+  </si>
+  <si>
+    <t>whipped cream</t>
+  </si>
+  <si>
+    <t>yeast</t>
+  </si>
+  <si>
+    <t>yellow mustard</t>
   </si>
 </sst>
 </file>
@@ -495,8 +555,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CD243A6-3128-45AE-AB78-995ED60CA29C}" name="Table1" displayName="Table1" ref="A1:A147" totalsRowShown="0" dataDxfId="1">
-  <autoFilter ref="A1:A147" xr:uid="{6CD243A6-3128-45AE-AB78-995ED60CA29C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CD243A6-3128-45AE-AB78-995ED60CA29C}" name="Table1" displayName="Table1" ref="A1:A148" totalsRowShown="0" dataDxfId="1">
+  <autoFilter ref="A1:A148" xr:uid="{6CD243A6-3128-45AE-AB78-995ED60CA29C}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{96714597-BB3B-4C97-ACBE-6770A363FEDB}" name="Ingredient" dataDxfId="0"/>
   </tableColumns>
@@ -801,7 +861,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66807D0D-95DD-48CD-972D-869D290E1F5D}">
-  <dimension ref="A1:A147"/>
+  <dimension ref="A1:A148"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46.85546875" customWidth="1"/>
@@ -814,695 +874,738 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>11</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>13</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>20</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>33</v>
+        <v>88</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>37</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>39</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>41</v>
+        <v>92</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>45</v>
+        <v>94</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>46</v>
+        <v>95</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>49</v>
+        <v>97</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>53</v>
+        <v>99</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>54</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>58</v>
+        <v>102</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>61</v>
+        <v>104</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>64</v>
+        <v>105</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>65</v>
+        <v>106</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>66</v>
+        <v>107</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>67</v>
+        <v>108</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>68</v>
+        <v>109</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>69</v>
+        <v>110</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>73</v>
+        <v>38</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>74</v>
+        <v>111</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>76</v>
+        <v>113</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>77</v>
+        <v>114</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>84</v>
+        <v>118</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>85</v>
+        <v>41</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>122</v>
+        <v>42</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>86</v>
+        <v>120</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>91</v>
+        <v>45</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>92</v>
+        <v>46</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>93</v>
+        <v>47</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>95</v>
+        <v>48</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
-        <v>97</v>
+        <v>49</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
-        <v>99</v>
+        <v>124</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
-        <v>100</v>
+        <v>52</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
-        <v>102</v>
+        <v>126</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
-        <v>105</v>
+        <v>53</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
-        <v>110</v>
+        <v>54</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
-        <v>111</v>
+        <v>55</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
-        <v>112</v>
+        <v>56</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
-        <v>113</v>
+        <v>57</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
-        <v>114</v>
+        <v>59</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
-        <v>115</v>
+        <v>58</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
-        <v>116</v>
+        <v>60</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
-        <v>118</v>
+        <v>61</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
-        <v>121</v>
+        <v>62</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
-        <v>125</v>
+        <v>63</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
-        <v>126</v>
+        <v>64</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A129" s="1"/>
+      <c r="A129" s="1" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A130" s="1"/>
+      <c r="A130" s="1" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A131" s="1"/>
+      <c r="A131" s="1" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A132" s="1"/>
+      <c r="A132" s="1" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A133" s="1"/>
+      <c r="A133" s="1" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A134" s="1"/>
+      <c r="A134" s="1" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A135" s="1"/>
+      <c r="A135" s="1" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A136" s="1"/>
+      <c r="A136" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A137" s="1"/>
+      <c r="A137" s="1" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A138" s="1"/>
+      <c r="A138" s="1" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A139" s="1"/>
+      <c r="A139" s="1" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A140" s="1"/>
+      <c r="A140" s="1" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A141" s="1"/>
+      <c r="A141" s="1" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A142" s="1"/>
+      <c r="A142" s="1" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A143" s="1"/>
+      <c r="A143" s="1" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A144" s="1"/>
+      <c r="A144" s="1" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A145" s="1"/>
+      <c r="A145" s="1" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A146" s="1"/>
+      <c r="A146" s="1" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A147" s="1"/>
+      <c r="A147" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A148" s="1" t="s">
+        <v>73</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>